<commit_message>
adding some analysis of training progress
</commit_message>
<xml_diff>
--- a/ecg_classification_model/training_progress.xlsx
+++ b/ecg_classification_model/training_progress.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/griffin/Documents/Data_Science_Projects/bhf_classification/ecg_classification_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE9EC581-E5E3-234B-B6ED-3968D609EEC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC095F02-9BBC-1F4A-AFA2-355DEEF9F2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1420" yWindow="760" windowWidth="28040" windowHeight="17440" xr2:uid="{91BACCCC-FC76-354F-B9A7-49FE9C42D7A7}"/>
   </bookViews>
@@ -134,9 +134,6 @@
     <t>[0.6403 0.4398 0.5579 0.5735 0.2933]</t>
   </si>
   <si>
-    <t>[ 0.6436 0.4295 0.5954 0.6070 0.1733]</t>
-  </si>
-  <si>
     <t>[0.5480 0.3965 0.6774 0.6647 0.2191]</t>
   </si>
   <si>
@@ -213,6 +210,9 @@
   </si>
   <si>
     <t>[0.6349 0.4800 0.5802 0.6438 0.1862</t>
+  </si>
+  <si>
+    <t>[0.6436 0.4295 0.5954 0.6070 0.1733]</t>
   </si>
 </sst>
 </file>
@@ -273,12 +273,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -711,7 +712,7 @@
         <v>0.1079</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F2" s="3">
         <v>0.39439999999999997</v>
@@ -723,10 +724,10 @@
         <v>8.3400000000000002E-2</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -743,7 +744,7 @@
         <v>0.16309999999999999</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F3" s="1">
         <v>0.35149999999999998</v>
@@ -755,7 +756,7 @@
         <v>0.2475</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>19</v>
@@ -775,7 +776,7 @@
         <v>0.20369999999999999</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F4" s="1">
         <v>0.38009999999999999</v>
@@ -787,7 +788,7 @@
         <v>0.29380000000000001</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>19</v>
@@ -807,7 +808,7 @@
         <v>0.25069999999999998</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5" s="1">
         <v>0.28970000000000001</v>
@@ -819,7 +820,7 @@
         <v>0.2984</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>19</v>
@@ -839,7 +840,7 @@
         <v>0.28410000000000002</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F6" s="1">
         <v>0.27810000000000001</v>
@@ -851,7 +852,7 @@
         <v>0.31879999999999997</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>19</v>
@@ -998,8 +999,8 @@
       <c r="D11" s="2">
         <v>0.29549999999999998</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>32</v>
+      <c r="E11" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="F11" s="2">
         <v>0.28589999999999999</v>
@@ -1011,7 +1012,7 @@
         <v>0.3372</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>19</v>
@@ -1031,7 +1032,7 @@
         <v>0.31130000000000002</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F12" s="2">
         <v>0.26140000000000002</v>
@@ -1043,7 +1044,7 @@
         <v>0.3513</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>19</v>
@@ -1255,7 +1256,7 @@
         <v>0.40400000000000003</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F19" s="2">
         <v>0.62770000000000004</v>
@@ -1267,7 +1268,7 @@
         <v>0.39350000000000002</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J19" s="1" t="s">
         <v>18</v>
@@ -1287,7 +1288,7 @@
         <v>0.38219999999999998</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F20" s="2">
         <v>0.745</v>
@@ -1299,7 +1300,7 @@
         <v>0.35589999999999999</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>19</v>
@@ -1319,7 +1320,7 @@
         <v>0.37419999999999998</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F21" s="2">
         <v>0.70099999999999996</v>
@@ -1331,7 +1332,7 @@
         <v>0.34499999999999997</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>19</v>
@@ -1351,7 +1352,7 @@
         <v>0.37859999999999999</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F22" s="2">
         <v>0.61350000000000005</v>
@@ -1363,7 +1364,7 @@
         <v>0.3876</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="J22" s="1" t="s">
         <v>19</v>
@@ -1383,7 +1384,7 @@
         <v>0.39100000000000001</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F23" s="2">
         <v>0.62390000000000001</v>
@@ -1395,7 +1396,7 @@
         <v>0.38179999999999997</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>19</v>
@@ -1415,7 +1416,7 @@
         <v>0.40699999999999997</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F24" s="2">
         <v>0.62609999999999999</v>
@@ -1427,7 +1428,7 @@
         <v>0.4002</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
update training progress xlsx
</commit_message>
<xml_diff>
--- a/ecg_classification_model/training_progress.xlsx
+++ b/ecg_classification_model/training_progress.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/griffin/Documents/Data_Science_Projects/bhf_classification/ecg_classification_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC095F02-9BBC-1F4A-AFA2-355DEEF9F2B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8B0A79-1572-8B42-9201-D8F90DB4C007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1420" yWindow="760" windowWidth="28040" windowHeight="17440" xr2:uid="{91BACCCC-FC76-354F-B9A7-49FE9C42D7A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="71">
   <si>
     <t>Epoch</t>
   </si>
@@ -213,13 +213,49 @@
   </si>
   <si>
     <t>[0.6436 0.4295 0.5954 0.6070 0.1733]</t>
+  </si>
+  <si>
+    <t>[0.7339 0.6170 0.7458 0.7243 0.5448]</t>
+  </si>
+  <si>
+    <t>[0.6598 0.4641 0.6799 0.6338 0.5221]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reset </t>
+  </si>
+  <si>
+    <t>[0.6254 0.5028 0.6868 0.6138 0.3962]</t>
+  </si>
+  <si>
+    <t>[0.7036 0.5641 0.7115 0.6913 0.5130]</t>
+  </si>
+  <si>
+    <t>[0.6418 0.4685 0.6593 0.6207 0.2664]</t>
+  </si>
+  <si>
+    <t>[0.6567 0.4268 0.7229 0.6778 0.4692]</t>
+  </si>
+  <si>
+    <t>[0.7477 0.6564 0.7584 0.7563 0.5533]</t>
+  </si>
+  <si>
+    <t>[0.7036 0.5071 0.7158 0.6670 0.5021]</t>
+  </si>
+  <si>
+    <t>[0.7789 0.6816 0.7998 0.7909 0.6044</t>
+  </si>
+  <si>
+    <t>[0.6806 0.4630 0.6961 0.6690 0.5174]</t>
+  </si>
+  <si>
+    <t>Reset, removed scheduler (just using lr=5e-4)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -252,6 +288,12 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF202124"/>
+      <name val="Courier New"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -279,7 +321,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -651,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FCDFC6-C99C-D343-998E-FFAC6AB50B7A}">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" customWidth="1"/>
@@ -999,7 +1041,7 @@
       <c r="D11" s="2">
         <v>0.29549999999999998</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" t="s">
         <v>58</v>
       </c>
       <c r="F11" s="2">
@@ -1432,6 +1474,206 @@
       </c>
       <c r="J24" s="1" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>29</v>
+      </c>
+      <c r="B25">
+        <v>0.4002</v>
+      </c>
+      <c r="C25">
+        <v>0.59550000000000003</v>
+      </c>
+      <c r="D25">
+        <v>0.4224</v>
+      </c>
+      <c r="E25" t="s">
+        <v>59</v>
+      </c>
+      <c r="F25">
+        <v>0.64470000000000005</v>
+      </c>
+      <c r="G25">
+        <v>0.49480000000000002</v>
+      </c>
+      <c r="H25">
+        <v>0.39560000000000001</v>
+      </c>
+      <c r="I25" t="s">
+        <v>60</v>
+      </c>
+      <c r="J25" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="19" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>30</v>
+      </c>
+      <c r="B26">
+        <v>0.48530000000000001</v>
+      </c>
+      <c r="C26">
+        <v>0.54310000000000003</v>
+      </c>
+      <c r="D26">
+        <v>0.39860000000000001</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" s="5">
+        <v>0.67290000000000005</v>
+      </c>
+      <c r="G26" s="5">
+        <v>0.47860000000000003</v>
+      </c>
+      <c r="H26" s="5">
+        <v>0.38400000000000001</v>
+      </c>
+      <c r="I26" t="s">
+        <v>62</v>
+      </c>
+      <c r="J26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>31</v>
+      </c>
+      <c r="B27">
+        <v>0.48</v>
+      </c>
+      <c r="C27">
+        <v>0.54039999999999999</v>
+      </c>
+      <c r="D27">
+        <v>0.39879999999999999</v>
+      </c>
+      <c r="E27" t="s">
+        <v>63</v>
+      </c>
+      <c r="F27">
+        <v>0.69350000000000001</v>
+      </c>
+      <c r="G27">
+        <v>0.39889999999999998</v>
+      </c>
+      <c r="H27">
+        <v>0.37440000000000001</v>
+      </c>
+      <c r="I27" t="s">
+        <v>64</v>
+      </c>
+      <c r="J27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>32</v>
+      </c>
+      <c r="B28">
+        <v>0.4234</v>
+      </c>
+      <c r="C28">
+        <v>0.57399999999999995</v>
+      </c>
+      <c r="D28">
+        <v>0.41460000000000002</v>
+      </c>
+      <c r="E28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28">
+        <v>0.66220000000000001</v>
+      </c>
+      <c r="G28">
+        <v>0.50439999999999996</v>
+      </c>
+      <c r="H28">
+        <v>0.3977</v>
+      </c>
+      <c r="I28" t="s">
+        <v>65</v>
+      </c>
+      <c r="J28" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>33</v>
+      </c>
+      <c r="B29">
+        <v>0.34749999999999998</v>
+      </c>
+      <c r="C29">
+        <v>0.63460000000000005</v>
+      </c>
+      <c r="D29">
+        <v>0.44059999999999999</v>
+      </c>
+      <c r="E29" t="s">
+        <v>66</v>
+      </c>
+      <c r="F29">
+        <v>0.73399999999999999</v>
+      </c>
+      <c r="G29">
+        <v>0.55859999999999999</v>
+      </c>
+      <c r="H29">
+        <v>0.40279999999999999</v>
+      </c>
+      <c r="I29" t="s">
+        <v>67</v>
+      </c>
+      <c r="J29" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>34</v>
+      </c>
+      <c r="B30">
+        <v>0.29239999999999999</v>
+      </c>
+      <c r="C30">
+        <v>0.68289999999999995</v>
+      </c>
+      <c r="D30">
+        <v>0.45950000000000002</v>
+      </c>
+      <c r="E30" t="s">
+        <v>68</v>
+      </c>
+      <c r="F30">
+        <v>0.78769999999999996</v>
+      </c>
+      <c r="G30">
+        <v>0.57050000000000001</v>
+      </c>
+      <c r="H30">
+        <v>0.39689999999999998</v>
+      </c>
+      <c r="I30" t="s">
+        <v>69</v>
+      </c>
+      <c r="J30" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>35</v>
+      </c>
+      <c r="J31" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>